<commit_message>
Excel files modification: SheetNames
</commit_message>
<xml_diff>
--- a/resources/Test_import.xlsx
+++ b/resources/Test_import.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B819B399-221D-4351-BD18-CFD2F0D35D2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFD9BAB-5EE5-44CD-BB27-10F7105CA9C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1848" yWindow="1944" windowWidth="17280" windowHeight="8880" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Parametres simulation" sheetId="1" r:id="rId1"/>
+    <sheet name="Profil digestion" sheetId="2" r:id="rId2"/>
+    <sheet name="Paramètre repas" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -56,16 +58,16 @@
     <t>Débit de transition</t>
   </si>
   <si>
-    <t>Nom du profil</t>
-  </si>
-  <si>
     <t>Test1</t>
   </si>
   <si>
     <t>Test2</t>
   </si>
   <si>
-    <t>Profil2</t>
+    <t>Nom de la config</t>
+  </si>
+  <si>
+    <t>config6</t>
   </si>
 </sst>
 </file>
@@ -521,7 +523,7 @@
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="1" max="1" width="14.21875" customWidth="1"/>
     <col min="2" max="2" width="21.33203125" customWidth="1"/>
     <col min="3" max="3" width="22.21875" customWidth="1"/>
     <col min="4" max="4" width="23.5546875" customWidth="1"/>
@@ -531,7 +533,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
@@ -551,7 +553,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" s="5">
         <v>20</v>
@@ -571,7 +573,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" s="5">
         <v>80</v>
@@ -636,4 +638,22 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{009CA921-60F2-474C-A0A4-508B81F79D12}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2271AA62-FFE6-4BEA-BC05-4E45C08DC32E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
problem fix + optimization
</commit_message>
<xml_diff>
--- a/resources/Test_import.xlsx
+++ b/resources/Test_import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA125DC-8EB7-4AE8-8338-A6EC164480D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46FB8E4A-2281-465D-93FB-2326EB4E4527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="3" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametres simulation" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Débit d'entrée enzyme</t>
   </si>
@@ -126,6 +126,12 @@
   </si>
   <si>
     <t>Taille (pouce)</t>
+  </si>
+  <si>
+    <t>Volume enzyme (ml)</t>
+  </si>
+  <si>
+    <t>Total particules</t>
   </si>
 </sst>
 </file>
@@ -246,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -259,7 +265,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -594,38 +599,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F695C7B3-19CB-4070-9BD5-C34B803C5B05}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" customWidth="1"/>
-    <col min="2" max="2" width="21.33203125" customWidth="1"/>
-    <col min="3" max="3" width="22.21875" customWidth="1"/>
-    <col min="4" max="4" width="23.5546875" customWidth="1"/>
-    <col min="5" max="5" width="14.109375" customWidth="1"/>
-    <col min="6" max="6" width="19.109375" customWidth="1"/>
+    <col min="2" max="2" width="21.21875" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" customWidth="1"/>
+    <col min="4" max="4" width="22.21875" customWidth="1"/>
+    <col min="5" max="5" width="23.5546875" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" customWidth="1"/>
+    <col min="7" max="7" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
@@ -633,81 +642,93 @@
         <v>20</v>
       </c>
       <c r="C2" s="5">
+        <v>20</v>
+      </c>
+      <c r="D2" s="5">
         <v>30</v>
       </c>
-      <c r="D2" s="5">
+      <c r="E2" s="5">
         <v>10000</v>
       </c>
-      <c r="E2" s="5">
+      <c r="F2" s="5">
         <v>60</v>
       </c>
-      <c r="F2" s="1">
+      <c r="G2" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="5">
+        <v>20</v>
+      </c>
+      <c r="C3" s="5">
         <v>80</v>
       </c>
-      <c r="C3" s="5">
+      <c r="D3" s="5">
         <v>100</v>
       </c>
-      <c r="D3" s="5">
+      <c r="E3" s="5">
         <v>10000</v>
       </c>
-      <c r="E3" s="5">
+      <c r="F3" s="5">
         <v>1</v>
       </c>
-      <c r="F3" s="1">
+      <c r="G3" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="5">
+        <v>20</v>
+      </c>
+      <c r="C4" s="5">
         <v>100</v>
       </c>
-      <c r="C4" s="5">
+      <c r="D4" s="5">
         <v>300</v>
       </c>
-      <c r="D4" s="5">
+      <c r="E4" s="5">
         <v>10000</v>
       </c>
-      <c r="E4" s="5">
+      <c r="F4" s="5">
         <v>10</v>
       </c>
-      <c r="F4" s="1">
+      <c r="G4" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F5" s="5"/>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="F6" s="5"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
-      <c r="F7" s="2"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1000,7 +1021,7 @@
       <c r="A2">
         <v>2.1</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2">
         <f>1/16</f>
         <v>6.25E-2</v>
       </c>
@@ -1012,7 +1033,7 @@
       <c r="A3">
         <v>2.1</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3">
         <f>3/32</f>
         <v>9.375E-2</v>
       </c>
@@ -1024,7 +1045,7 @@
       <c r="A4">
         <v>2.1</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4">
         <f>1/8</f>
         <v>0.125</v>
       </c>
@@ -1036,7 +1057,7 @@
       <c r="A5">
         <v>2.1</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5">
         <f>5/32</f>
         <v>0.15625</v>
       </c>
@@ -1048,7 +1069,7 @@
       <c r="A6">
         <v>0.9</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6">
         <f>1/16</f>
         <v>6.25E-2</v>
       </c>
@@ -1060,7 +1081,7 @@
       <c r="A7">
         <v>0.9</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7">
         <f>3/32</f>
         <v>9.375E-2</v>
       </c>
@@ -1072,7 +1093,7 @@
       <c r="A8">
         <v>0.9</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8">
         <f>1/8</f>
         <v>0.125</v>
       </c>
@@ -1084,7 +1105,7 @@
       <c r="A9">
         <v>0.9</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9">
         <f>5/32</f>
         <v>0.15625</v>
       </c>
@@ -1096,7 +1117,7 @@
       <c r="A10">
         <v>1.1399999999999999</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10">
         <f>1/16</f>
         <v>6.25E-2</v>
       </c>
@@ -1108,7 +1129,7 @@
       <c r="A11">
         <v>1.1399999999999999</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11">
         <f>3/32</f>
         <v>9.375E-2</v>
       </c>
@@ -1120,7 +1141,7 @@
       <c r="A12">
         <v>1.1399999999999999</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12">
         <f>1/8</f>
         <v>0.125</v>
       </c>
@@ -1132,7 +1153,7 @@
       <c r="A13">
         <v>1.1399999999999999</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13">
         <f>5/32</f>
         <v>0.15625</v>
       </c>
@@ -1144,7 +1165,7 @@
       <c r="A14">
         <v>0.98</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14">
         <f>1/16</f>
         <v>6.25E-2</v>
       </c>
@@ -1156,7 +1177,7 @@
       <c r="A15">
         <v>0.98</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15">
         <f>3/32</f>
         <v>9.375E-2</v>
       </c>
@@ -1168,7 +1189,7 @@
       <c r="A16">
         <v>0.98</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16">
         <f>1/8</f>
         <v>0.125</v>
       </c>
@@ -1180,7 +1201,7 @@
       <c r="A17">
         <v>0.98</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17">
         <f>5/32</f>
         <v>0.15625</v>
       </c>
@@ -1195,16 +1216,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2271AA62-FFE6-4BEA-BC05-4E45C08DC32E}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="17.5546875" customWidth="1"/>
     <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>19</v>
       </c>
@@ -1220,8 +1242,11 @@
       <c r="E1" s="4" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
         <v>200</v>
       </c>
@@ -1237,118 +1262,138 @@
       <c r="E2" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" s="1">
+        <f>SUM(Particules!C1:C100)</f>
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
       <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
       <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="1"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="1"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
       <c r="E17" s="1"/>
-    </row>
-    <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
       <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Increment 3.1 and 3.2 : Particle motion and flow
</commit_message>
<xml_diff>
--- a/resources/Test_import.xlsx
+++ b/resources/Test_import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46FB8E4A-2281-465D-93FB-2326EB4E4527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8942E5CF-AE47-4F7A-B28B-CDC17021B647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="3" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
+    <workbookView xWindow="1848" yWindow="1944" windowWidth="17280" windowHeight="8880" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametres simulation" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Débit d'entrée enzyme</t>
   </si>
@@ -65,13 +65,7 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>Test2</t>
-  </si>
-  <si>
     <t>Nom de la config</t>
-  </si>
-  <si>
-    <t>config6</t>
   </si>
   <si>
     <t>Débit du va et vient</t>
@@ -613,10 +607,10 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>0</v>
@@ -648,60 +642,32 @@
         <v>30</v>
       </c>
       <c r="E2" s="5">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="F2" s="5">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="G2" s="1">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="5">
-        <v>20</v>
-      </c>
-      <c r="C3" s="5">
-        <v>80</v>
-      </c>
-      <c r="D3" s="5">
-        <v>100</v>
-      </c>
-      <c r="E3" s="5">
-        <v>10000</v>
-      </c>
-      <c r="F3" s="5">
-        <v>1</v>
-      </c>
-      <c r="G3" s="1">
-        <v>10</v>
-      </c>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="5">
-        <v>20</v>
-      </c>
-      <c r="C4" s="5">
-        <v>100</v>
-      </c>
-      <c r="D4" s="5">
-        <v>300</v>
-      </c>
-      <c r="E4" s="5">
-        <v>10000</v>
-      </c>
-      <c r="F4" s="5">
-        <v>10</v>
-      </c>
-      <c r="G4" s="1">
-        <v>5</v>
-      </c>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
@@ -757,33 +723,33 @@
         <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B2" s="8">
         <v>2</v>
@@ -812,7 +778,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B3" s="5">
         <v>10</v>
@@ -1008,13 +974,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="B1" t="s">
-        <v>27</v>
-      </c>
       <c r="C1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -1038,7 +1004,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="C3">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1050,7 +1016,7 @@
         <v>0.125</v>
       </c>
       <c r="C4">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1062,7 +1028,7 @@
         <v>0.15625</v>
       </c>
       <c r="C5">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1086,7 +1052,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="C7">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1098,7 +1064,7 @@
         <v>0.125</v>
       </c>
       <c r="C8">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1110,7 +1076,7 @@
         <v>0.15625</v>
       </c>
       <c r="C9">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -1134,7 +1100,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="C11">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1146,7 +1112,7 @@
         <v>0.125</v>
       </c>
       <c r="C12">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1158,7 +1124,7 @@
         <v>0.15625</v>
       </c>
       <c r="C13">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1182,7 +1148,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="C15">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -1194,7 +1160,7 @@
         <v>0.125</v>
       </c>
       <c r="C16">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1206,7 +1172,7 @@
         <v>0.15625</v>
       </c>
       <c r="C17">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1228,22 +1194,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>23</v>
-      </c>
       <c r="F1" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1264,7 +1230,7 @@
       </c>
       <c r="F2" s="1">
         <f>SUM(Particules!C1:C100)</f>
-        <v>560</v>
+        <v>320</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
3.3 + 3.4 : Archimedes + settling calculation
</commit_message>
<xml_diff>
--- a/resources/Test_import.xlsx
+++ b/resources/Test_import.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2343754-AF72-469E-9CA7-7BE561D229D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36EDD5BF-74ED-4206-82F9-850D413B33EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1848" yWindow="1944" windowWidth="17340" windowHeight="8880" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametres simulation" sheetId="1" r:id="rId1"/>
     <sheet name="Profil digestion" sheetId="2" r:id="rId2"/>
     <sheet name="Particules" sheetId="4" r:id="rId3"/>
-    <sheet name="Parametres repas" sheetId="3" r:id="rId4"/>
+    <sheet name="Feuil1" sheetId="5" r:id="rId4"/>
+    <sheet name="Parametres repas" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Débit d'entrée enzyme</t>
   </si>
@@ -126,6 +127,9 @@
   </si>
   <si>
     <t>Total particules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tests sur les particules </t>
   </si>
 </sst>
 </file>
@@ -642,7 +646,7 @@
         <v>30</v>
       </c>
       <c r="E2" s="5">
-        <v>20000</v>
+        <v>30000</v>
       </c>
       <c r="F2" s="5">
         <v>1</v>
@@ -970,6 +974,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.88671875" customWidth="1"/>
+    <col min="5" max="6" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -985,194 +990,194 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2.1</v>
+        <v>2100</v>
       </c>
       <c r="B2">
         <f>1/16</f>
         <v>6.25E-2</v>
       </c>
       <c r="C2">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>2.1</v>
+        <v>2100</v>
       </c>
       <c r="B3">
         <f>3/32</f>
         <v>9.375E-2</v>
       </c>
       <c r="C3">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>2.1</v>
+        <v>2100</v>
       </c>
       <c r="B4">
         <f>1/8</f>
         <v>0.125</v>
       </c>
       <c r="C4">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>2.1</v>
+        <v>2100</v>
       </c>
       <c r="B5">
         <f>5/32</f>
         <v>0.15625</v>
       </c>
       <c r="C5">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.9</v>
+        <v>900</v>
       </c>
       <c r="B6">
         <f>1/16</f>
         <v>6.25E-2</v>
       </c>
       <c r="C6">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.9</v>
+        <v>900</v>
       </c>
       <c r="B7">
         <f>3/32</f>
         <v>9.375E-2</v>
       </c>
       <c r="C7">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.9</v>
+        <v>900</v>
       </c>
       <c r="B8">
         <f>1/8</f>
         <v>0.125</v>
       </c>
       <c r="C8">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.9</v>
+        <v>900</v>
       </c>
       <c r="B9">
         <f>5/32</f>
         <v>0.15625</v>
       </c>
       <c r="C9">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1.1399999999999999</v>
+        <v>1140</v>
       </c>
       <c r="B10">
         <f>1/16</f>
         <v>6.25E-2</v>
       </c>
       <c r="C10">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1.1399999999999999</v>
+        <v>1140</v>
       </c>
       <c r="B11">
         <f>3/32</f>
         <v>9.375E-2</v>
       </c>
       <c r="C11">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1.1399999999999999</v>
+        <v>1140</v>
       </c>
       <c r="B12">
         <f>1/8</f>
         <v>0.125</v>
       </c>
       <c r="C12">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1.1399999999999999</v>
+        <v>1140</v>
       </c>
       <c r="B13">
         <f>5/32</f>
         <v>0.15625</v>
       </c>
       <c r="C13">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>0.98</v>
+        <v>980</v>
       </c>
       <c r="B14">
         <f>1/16</f>
         <v>6.25E-2</v>
       </c>
       <c r="C14">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>0.98</v>
+        <v>980</v>
       </c>
       <c r="B15">
         <f>3/32</f>
         <v>9.375E-2</v>
       </c>
       <c r="C15">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>0.98</v>
+        <v>980</v>
       </c>
       <c r="B16">
         <f>1/8</f>
         <v>0.125</v>
       </c>
       <c r="C16">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>0.98</v>
+        <v>980</v>
       </c>
       <c r="B17">
         <f>5/32</f>
         <v>0.15625</v>
       </c>
       <c r="C17">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1181,6 +1186,213 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{374F7619-311F-47F6-BC63-15F51184BE61}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2100</v>
+      </c>
+      <c r="B2">
+        <f>1/16</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="C2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2100</v>
+      </c>
+      <c r="B3">
+        <f>3/32</f>
+        <v>9.375E-2</v>
+      </c>
+      <c r="C3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2100</v>
+      </c>
+      <c r="B4">
+        <f>1/8</f>
+        <v>0.125</v>
+      </c>
+      <c r="C4">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2100</v>
+      </c>
+      <c r="B5">
+        <f>5/32</f>
+        <v>0.15625</v>
+      </c>
+      <c r="C5">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>900</v>
+      </c>
+      <c r="B6">
+        <f>1/16</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="C6">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>900</v>
+      </c>
+      <c r="B7">
+        <f>3/32</f>
+        <v>9.375E-2</v>
+      </c>
+      <c r="C7">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>900</v>
+      </c>
+      <c r="B8">
+        <f>1/8</f>
+        <v>0.125</v>
+      </c>
+      <c r="C8">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>900</v>
+      </c>
+      <c r="B9">
+        <f>5/32</f>
+        <v>0.15625</v>
+      </c>
+      <c r="C9">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1140</v>
+      </c>
+      <c r="B10">
+        <f>1/16</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="C10">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1140</v>
+      </c>
+      <c r="B11">
+        <f>3/32</f>
+        <v>9.375E-2</v>
+      </c>
+      <c r="C11">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>1140</v>
+      </c>
+      <c r="B12">
+        <f>1/8</f>
+        <v>0.125</v>
+      </c>
+      <c r="C12">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1140</v>
+      </c>
+      <c r="B13">
+        <f>5/32</f>
+        <v>0.15625</v>
+      </c>
+      <c r="C13">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>980</v>
+      </c>
+      <c r="B14">
+        <f>1/16</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="C14">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>980</v>
+      </c>
+      <c r="B15">
+        <f>3/32</f>
+        <v>9.375E-2</v>
+      </c>
+      <c r="C15">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>980</v>
+      </c>
+      <c r="B16">
+        <f>1/8</f>
+        <v>0.125</v>
+      </c>
+      <c r="C16">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>980</v>
+      </c>
+      <c r="B17">
+        <f>5/32</f>
+        <v>0.15625</v>
+      </c>
+      <c r="C17">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2271AA62-FFE6-4BEA-BC05-4E45C08DC32E}">
   <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1230,7 +1442,7 @@
       </c>
       <c r="F2" s="1">
         <f>SUM(Particules!C1:C100)</f>
-        <v>320</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Increment 3.6 : residence time distribution calculation
</commit_message>
<xml_diff>
--- a/resources/Test_import.xlsx
+++ b/resources/Test_import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36EDD5BF-74ED-4206-82F9-850D413B33EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A093210D-1CE6-4A94-B3A2-3C64BEC6FCD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
+    <workbookView xWindow="1848" yWindow="1944" windowWidth="17340" windowHeight="8880" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametres simulation" sheetId="1" r:id="rId1"/>
@@ -646,7 +646,7 @@
         <v>30</v>
       </c>
       <c r="E2" s="5">
-        <v>30000</v>
+        <v>43200</v>
       </c>
       <c r="F2" s="5">
         <v>1</v>
@@ -997,7 +997,7 @@
         <v>6.25E-2</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1009,7 +1009,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="C3">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1021,7 +1021,7 @@
         <v>0.125</v>
       </c>
       <c r="C4">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1033,7 +1033,7 @@
         <v>0.15625</v>
       </c>
       <c r="C5">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1045,7 +1045,7 @@
         <v>6.25E-2</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1057,7 +1057,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="C7">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1069,7 +1069,7 @@
         <v>0.125</v>
       </c>
       <c r="C8">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1081,7 +1081,7 @@
         <v>0.15625</v>
       </c>
       <c r="C9">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -1093,7 +1093,7 @@
         <v>6.25E-2</v>
       </c>
       <c r="C10">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -1105,7 +1105,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="C11">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1117,7 +1117,7 @@
         <v>0.125</v>
       </c>
       <c r="C12">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1129,7 +1129,7 @@
         <v>0.15625</v>
       </c>
       <c r="C13">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1141,7 +1141,7 @@
         <v>6.25E-2</v>
       </c>
       <c r="C14">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -1153,7 +1153,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="C15">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -1165,7 +1165,7 @@
         <v>0.125</v>
       </c>
       <c r="C16">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1177,7 +1177,7 @@
         <v>0.15625</v>
       </c>
       <c r="C17">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="F2" s="1">
         <f>SUM(Particules!C1:C100)</f>
-        <v>160</v>
+        <v>480</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
GUI optimization + bug fixes
</commit_message>
<xml_diff>
--- a/resources/Test_import.xlsx
+++ b/resources/Test_import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A093210D-1CE6-4A94-B3A2-3C64BEC6FCD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FDE364A-5F5A-4922-B8C4-181C277B9C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1848" yWindow="1944" windowWidth="17340" windowHeight="8880" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
+    <workbookView xWindow="1848" yWindow="1944" windowWidth="9912" windowHeight="8880" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametres simulation" sheetId="1" r:id="rId1"/>
@@ -637,13 +637,13 @@
         <v>6</v>
       </c>
       <c r="B2" s="5">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C2" s="5">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D2" s="5">
-        <v>30</v>
+        <v>7200</v>
       </c>
       <c r="E2" s="5">
         <v>43200</v>
@@ -652,7 +652,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -1426,10 +1426,10 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
-        <v>200</v>
+        <v>30</v>
       </c>
       <c r="B2" s="8">
-        <v>10</v>
+        <v>900</v>
       </c>
       <c r="C2" s="9">
         <v>1.0000000000000001E-5</v>
@@ -1438,7 +1438,7 @@
         <v>0.98</v>
       </c>
       <c r="E2" s="1">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F2" s="1">
         <f>SUM(Particules!C1:C100)</f>

</xml_diff>

<commit_message>
adding spyder kernel lib to .venv
</commit_message>
<xml_diff>
--- a/resources/Test_import.xlsx
+++ b/resources/Test_import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE24955-2696-40DD-9215-D8E817D702DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288700A4-0855-4C6E-BD9A-1B4C266F6D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametres simulation" sheetId="1" r:id="rId1"/>
@@ -642,7 +642,7 @@
         <v>7200</v>
       </c>
       <c r="E2" s="5">
-        <v>20000</v>
+        <v>25000</v>
       </c>
       <c r="F2" s="5">
         <v>10</v>
@@ -966,7 +966,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{435F0B4B-A19D-4754-B1A7-C90AD7791F67}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.88671875" customWidth="1"/>
@@ -986,194 +986,14 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2100</v>
+        <v>1140</v>
       </c>
       <c r="B2">
-        <f>1/16</f>
-        <v>6.25E-2</v>
-      </c>
-      <c r="C2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2100</v>
-      </c>
-      <c r="B3">
         <f>3/32</f>
         <v>9.375E-2</v>
       </c>
-      <c r="C3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>2100</v>
-      </c>
-      <c r="B4">
-        <f>1/8</f>
-        <v>0.125</v>
-      </c>
-      <c r="C4">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>2100</v>
-      </c>
-      <c r="B5">
-        <f>5/32</f>
-        <v>0.15625</v>
-      </c>
-      <c r="C5">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>900</v>
-      </c>
-      <c r="B6">
-        <f>1/16</f>
-        <v>6.25E-2</v>
-      </c>
-      <c r="C6">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>900</v>
-      </c>
-      <c r="B7">
-        <f>3/32</f>
-        <v>9.375E-2</v>
-      </c>
-      <c r="C7">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>900</v>
-      </c>
-      <c r="B8">
-        <f>1/8</f>
-        <v>0.125</v>
-      </c>
-      <c r="C8">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>900</v>
-      </c>
-      <c r="B9">
-        <f>5/32</f>
-        <v>0.15625</v>
-      </c>
-      <c r="C9">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>1140</v>
-      </c>
-      <c r="B10">
-        <f>1/16</f>
-        <v>6.25E-2</v>
-      </c>
-      <c r="C10">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>1140</v>
-      </c>
-      <c r="B11">
-        <f>3/32</f>
-        <v>9.375E-2</v>
-      </c>
-      <c r="C11">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>1140</v>
-      </c>
-      <c r="B12">
-        <f>1/8</f>
-        <v>0.125</v>
-      </c>
-      <c r="C12">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>1140</v>
-      </c>
-      <c r="B13">
-        <f>5/32</f>
-        <v>0.15625</v>
-      </c>
-      <c r="C13">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>980</v>
-      </c>
-      <c r="B14">
-        <f>1/16</f>
-        <v>6.25E-2</v>
-      </c>
-      <c r="C14">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>980</v>
-      </c>
-      <c r="B15">
-        <f>3/32</f>
-        <v>9.375E-2</v>
-      </c>
-      <c r="C15">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>980</v>
-      </c>
-      <c r="B16">
-        <f>1/8</f>
-        <v>0.125</v>
-      </c>
-      <c r="C16">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>980</v>
-      </c>
-      <c r="B17">
-        <f>5/32</f>
-        <v>0.15625</v>
-      </c>
-      <c r="C17">
-        <v>30</v>
+      <c r="C2">
+        <v>1700</v>
       </c>
     </row>
   </sheetData>
@@ -1231,7 +1051,7 @@
       </c>
       <c r="F2" s="1">
         <f>SUM(Particules!C1:C100)</f>
-        <v>480</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Excel export: init + bug fixes on volume management
</commit_message>
<xml_diff>
--- a/resources/Test_import.xlsx
+++ b/resources/Test_import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\Canada\UdS\Projet\RTD_Modelisation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288700A4-0855-4C6E-BD9A-1B4C266F6D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E845FFE-8859-4297-8A2D-54E54FEEC16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{7BB19622-49C4-4242-B1EB-865F42CFBC30}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametres simulation" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Débit d'entrée enzyme</t>
   </si>
@@ -99,12 +99,6 @@
   </si>
   <si>
     <t>Période d'entrée de repas</t>
-  </si>
-  <si>
-    <t>Taille des particules</t>
-  </si>
-  <si>
-    <t>Densité des particules</t>
   </si>
   <si>
     <t>Viscosité</t>
@@ -246,7 +240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -258,7 +252,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -610,7 +603,7 @@
         <v>7</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>0</v>
@@ -645,7 +638,7 @@
         <v>25000</v>
       </c>
       <c r="F2" s="5">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G2" s="1">
         <v>4</v>
@@ -729,7 +722,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>13</v>
@@ -966,22 +959,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{435F0B4B-A19D-4754-B1A7-C90AD7791F67}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.88671875" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" t="s">
         <v>23</v>
       </c>
-      <c r="B1" t="s">
-        <v>25</v>
-      </c>
       <c r="C1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -989,11 +983,47 @@
         <v>1140</v>
       </c>
       <c r="B2">
+        <f>1/16</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="C2">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1140</v>
+      </c>
+      <c r="B3">
         <f>3/32</f>
         <v>9.375E-2</v>
       </c>
-      <c r="C2">
+      <c r="C3">
         <v>1700</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1140</v>
+      </c>
+      <c r="B4">
+        <f>1/8</f>
+        <v>0.125</v>
+      </c>
+      <c r="C4">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1140</v>
+      </c>
+      <c r="B5">
+        <f>5/32</f>
+        <v>0.15625</v>
+      </c>
+      <c r="C5">
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -1003,17 +1033,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2271AA62-FFE6-4BEA-BC05-4E45C08DC32E}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" customWidth="1"/>
-    <col min="4" max="4" width="19" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>17</v>
       </c>
@@ -1024,163 +1052,119 @@
         <v>19</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
         <v>30</v>
       </c>
       <c r="B2" s="8">
         <v>900</v>
       </c>
-      <c r="C2" s="9">
-        <v>1.0000000000000001E-5</v>
-      </c>
-      <c r="D2" s="8">
-        <v>0.98</v>
-      </c>
-      <c r="E2" s="1">
+      <c r="C2" s="1">
         <v>0.1</v>
       </c>
-      <c r="F2" s="1">
+      <c r="D2" s="1">
         <f>SUM(Particules!C1:C100)</f>
-        <v>1700</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>4300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+    </row>
+    <row r="18" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>